<commit_message>
added manually coded dataset, classifier, changed french press releases to only contain responses without questions, etc etc
</commit_message>
<xml_diff>
--- a/data/raw/council_minutes_data.xlsx
+++ b/data/raw/council_minutes_data.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wikto\python_project\EU_leadership_docs\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DB1E1A3-9603-40C9-B541-A8512B89074E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67F5A183-6F32-4BB1-980D-A740C5E5AE85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13970" windowHeight="10450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>